<commit_message>
modification de la matrice
</commit_message>
<xml_diff>
--- a/Matrice des tâches.xlsx
+++ b/Matrice des tâches.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="31">
   <si>
     <t xml:space="preserve">Matrice de répartition de charges (à remplir à chaque séance)</t>
   </si>
@@ -100,7 +100,19 @@
     <t xml:space="preserve">Correction pour passer de sfml 2 a 3</t>
   </si>
   <si>
-    <t xml:space="preserve">1h </t>
+    <t xml:space="preserve">30min </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Code 1,2 conversion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Code 1,2 debug</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Formule 1,2</t>
   </si>
 </sst>
 </file>
@@ -208,44 +220,48 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -438,226 +454,263 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="17.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="31.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="0" width="9.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="31.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="1" width="9.11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2"/>
+      <c r="A4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="G7" s="5"/>
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="G7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C8" s="5"/>
-      <c r="G8" s="5"/>
+      <c r="C8" s="6"/>
+      <c r="G8" s="6"/>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G13" s="5"/>
+      <c r="G13" s="6"/>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="G14" s="5"/>
+      <c r="G14" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="1" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="0" t="s">
+      <c r="B18" s="1" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
+      <c r="A20" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B20" s="6" t="n">
+      <c r="B20" s="7" t="n">
         <v>46274</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2"/>
+      <c r="A21" s="3"/>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="C22" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="E22" s="7" t="s">
+      <c r="E22" s="8" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="8" t="s">
+      <c r="B23" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="C23" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="8" t="s">
+      <c r="D23" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="E23" s="8"/>
+      <c r="E23" s="9"/>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="C24" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="D24" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="E24" s="8"/>
+      <c r="E24" s="9"/>
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D25" s="8" t="s">
+      <c r="D25" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="E25" s="8"/>
+      <c r="E25" s="9"/>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="C26" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="D26" s="9" t="s">
+      <c r="D26" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="E26" s="4"/>
+      <c r="E26" s="5"/>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="4"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
+      <c r="B27" s="5"/>
+      <c r="C27" s="5"/>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="8"/>
-      <c r="C28" s="8"/>
-      <c r="D28" s="8"/>
-      <c r="E28" s="8"/>
+      <c r="B28" s="9"/>
+      <c r="C28" s="9"/>
+      <c r="D28" s="9"/>
+      <c r="E28" s="9"/>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="2" t="s">
+      <c r="A30" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B30" s="6" t="n">
+      <c r="B30" s="7" t="n">
         <v>46275</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="2"/>
+      <c r="A31" s="3"/>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="C32" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="D32" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E32" s="2" t="s">
+      <c r="E32" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="0" t="s">
+    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B33" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C33" s="0" t="s">
+      <c r="C33" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="D33" s="0" t="s">
+      <c r="D33" s="9" t="s">
         <v>26</v>
       </c>
+      <c r="E33" s="9"/>
+    </row>
+    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C34" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E34" s="9"/>
+    </row>
+    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B35" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D35" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="E35" s="9"/>
+    </row>
+    <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B36" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C36" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="E36" s="9"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>